<commit_message>
Updated Fine Grain REPO
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -4,21 +4,21 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="108" windowWidth="22980" windowHeight="9288" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="108" windowWidth="22980" windowHeight="9288" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="simple" sheetId="1" r:id="rId1"/>
     <sheet name="hops" sheetId="2" r:id="rId2"/>
     <sheet name="Typo" sheetId="3" r:id="rId3"/>
     <sheet name="Vector" sheetId="4" r:id="rId4"/>
-    <sheet name="Tools" sheetId="5" r:id="rId5"/>
+    <sheet name="simple math question" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
   <si>
     <t>Question</t>
   </si>
@@ -388,9 +388,6 @@
     </r>
   </si>
   <si>
-    <t>What is the supplier name for the contract linked to the purchase order about “global data center infrastucture services”?</t>
-  </si>
-  <si>
     <t>Which purchase order is related to “cybersecurty monitoring services” and what are its payment terms?</t>
   </si>
   <si>
@@ -468,6 +465,310 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">What percentage of PurchaseOrders are marked </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>high_risk = YES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t>The payment terms for PO-INF-002 are **NET 45**.</t>
+  </si>
+  <si>
+    <t>The currency of PO-INF-006 is USD.</t>
+  </si>
+  <si>
+    <t>The total cost amount of PO-INF-003 is 1,600,000 USD.</t>
+  </si>
+  <si>
+    <r>
+      <t>The invoice number generated for PO-INF-001 is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>INV-001</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The approval status of PR-INF-003 is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>APPROVED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The contract agreement name linked to PO-INF-001 is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Global Data Center SLA."</t>
+    </r>
+  </si>
+  <si>
+    <t>Actual connection</t>
+  </si>
+  <si>
+    <t>(PurchaseOrder → Contract)</t>
+  </si>
+  <si>
+    <t>(PurchaseOrder → Contract → supplier_name)</t>
+  </si>
+  <si>
+    <t>(PurchaseOrder → Invoice)</t>
+  </si>
+  <si>
+    <t>(PurchaseOrder → PurchaseRequest)</t>
+  </si>
+  <si>
+    <r>
+      <t>The supplier name for the contract associated with PO-INF-008 is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>SecureCore Systems</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>I don’t know the invoice gross amount for the invoice generated from PO-INF-006 based on the provided information.</t>
+  </si>
+  <si>
+    <t>Original Question</t>
+  </si>
+  <si>
+    <t>Semantically Different word</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Which purchase order is for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>threat detection</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>security breach handling</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Original Question Response </t>
+  </si>
+  <si>
+    <t>Semantic Response</t>
+  </si>
+  <si>
+    <r>
+      <t>The approver name of the purchase request fulfilled by PO-INF-002 is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>MGR-INF-02</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>The purchase requisition title for the requisition fulfilled by PO-INF-010 is: "Identity and access management enhancement for privileged accounts."</t>
+  </si>
+  <si>
+    <t>Which contract talks about backup and disaster recovery with quarterly DR drills and penalties?</t>
+  </si>
+  <si>
+    <t>Which agreement covers data recovery planning, regular recovery testing, and financial consequences for failures?</t>
+  </si>
+  <si>
+    <t>Which purchase order supports global SD-WAN expansion to improve latency and resilience?</t>
+  </si>
+  <si>
+    <t>Which purchase order is about WAN network modernization to reduce delay and improve stability?</t>
+  </si>
+  <si>
+    <t>Which contract governs managed cloud services for AWS and Azure with RTO/RPO requirements?</t>
+  </si>
+  <si>
+    <t>Which agreement covers cloud operations support with recovery time and recovery point targets?</t>
+  </si>
+  <si>
+    <t>Which purchase order supports infrastructure observability tooling for real-time metrics, alerting, and root-cause analysis?</t>
+  </si>
+  <si>
+    <t>Which purchase order is about system monitoring tools that provide live performance tracking, alerts, and issue diagnosis?</t>
+  </si>
+  <si>
+    <r>
+      <t>The purchase order related to “cybersecurity monitoring services” is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PO-INF-003</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, and its payment terms are </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>NET 30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate Cypher query </t>
+  </si>
+  <si>
+    <t>MATCH (n:PurchaseOrder) WHERE toLower(n.line_item_description) CONTAINS toLower("cybersecurty monitoring services") RETURN n LIMIT 5</t>
+  </si>
+  <si>
+    <t>who is the supllier tied to the contrct for backup and disastor recovry?</t>
+  </si>
+  <si>
+    <t>The supplier tied to the contract for backup and disaster recovery (contract number C-INF-008 / PO-INF-004) is: Supplier ID: SUP-008</t>
+  </si>
+  <si>
+    <t>MATCH (n:Contract) WHERE toLower(n.agreement_name) CONTAINS toLower("backup and disaster recovery") RETURN n LIMIT 5</t>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">What is the </t>
     </r>
     <r>
@@ -479,7 +780,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>average total_cost_amount</t>
+      <t>average total cost amount</t>
     </r>
     <r>
       <rPr>
@@ -526,7 +827,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>total gross_amount</t>
+      <t>total gross amount</t>
     </r>
     <r>
       <rPr>
@@ -594,7 +895,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>invoice gross_amount</t>
+      <t>invoice gross amount</t>
     </r>
     <r>
       <rPr>
@@ -608,6 +909,9 @@
     </r>
   </si>
   <si>
+    <t>The highest invoice gross amount is 400000 and the lowest is 210000, so the difference is 190000.</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">What is the </t>
     </r>
@@ -620,7 +924,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>sum of total_cost_amount</t>
+      <t>sum of total cost amount</t>
     </r>
     <r>
       <rPr>
@@ -656,57 +960,19 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">What percentage of PurchaseOrders are marked </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+      <t>100% of the PurchaseOrders in the provided data are marked </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8.25"/>
+        <color rgb="FF158237"/>
+        <rFont val="Source Code Pro"/>
+        <family val="3"/>
       </rPr>
       <t>high_risk = YES</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>?</t>
-    </r>
-  </si>
-  <si>
-    <t>Response</t>
-  </si>
-  <si>
-    <t>The payment terms for PO-INF-002 are **NET 45**.</t>
-  </si>
-  <si>
-    <t>The currency of PO-INF-006 is USD.</t>
-  </si>
-  <si>
-    <t>The total cost amount of PO-INF-003 is 1,600,000 USD.</t>
-  </si>
-  <si>
-    <r>
-      <t>The invoice number generated for PO-INF-001 is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>INV-001</t>
-    </r>
-    <r>
-      <rPr>
         <sz val="10"/>
         <color rgb="FF31333F"/>
         <rFont val="Arial"/>
@@ -717,16 +983,34 @@
   </si>
   <si>
     <r>
-      <t>The approval status of PR-INF-003 is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>APPROVED</t>
+      <t>The total spend of all PurchaseOrders with payment terms </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>NET 30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>USD 10,300,000</t>
     </r>
     <r>
       <rPr>
@@ -740,45 +1024,34 @@
   </si>
   <si>
     <r>
-      <t>The contract agreement name linked to PO-INF-001 is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Global Data Center SLA."</t>
-    </r>
-  </si>
-  <si>
-    <t>Actual connection</t>
-  </si>
-  <si>
-    <t>(PurchaseOrder → Contract)</t>
-  </si>
-  <si>
-    <t>(PurchaseOrder → Contract → supplier_name)</t>
-  </si>
-  <si>
-    <t>(PurchaseOrder → Invoice)</t>
-  </si>
-  <si>
-    <t>(PurchaseOrder → PurchaseRequest)</t>
-  </si>
-  <si>
-    <r>
-      <t>The supplier name for the contract associated with PO-INF-008 is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>SecureCore Systems</t>
+      <t>The average total cost amount of all PurchaseOrders where </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8.25"/>
+        <color rgb="FF158237"/>
+        <rFont val="Source Code Pro"/>
+        <family val="3"/>
+      </rPr>
+      <t>high_risk = YES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>USD 2,900,000</t>
     </r>
     <r>
       <rPr>
@@ -791,79 +1064,17 @@
     </r>
   </si>
   <si>
-    <t>I don’t know the invoice gross amount for the invoice generated from PO-INF-006 based on the provided information.</t>
-  </si>
-  <si>
-    <t>Original Question</t>
-  </si>
-  <si>
-    <t>Semantically Different word</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Which purchase order is for </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>threat detection</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>security breach handling</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>?</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Original Question Response </t>
-  </si>
-  <si>
-    <t>Semantic Response</t>
-  </si>
-  <si>
-    <r>
-      <t>The approver name of the purchase request fulfilled by PO-INF-002 is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>MGR-INF-02</t>
+    <r>
+      <t>The sum of the total cost amount of all CAPEX purchase orders is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>USD 7,800,000</t>
     </r>
     <r>
       <rPr>
@@ -876,38 +1087,26 @@
     </r>
   </si>
   <si>
-    <t>The purchase requisition title for the requisition fulfilled by PO-INF-010 is: "Identity and access management enhancement for privileged accounts."</t>
-  </si>
-  <si>
-    <t>Which contract talks about backup and disaster recovery with quarterly DR drills and penalties?</t>
-  </si>
-  <si>
-    <t>Which agreement covers data recovery planning, regular recovery testing, and financial consequences for failures?</t>
-  </si>
-  <si>
-    <t>Which purchase order supports global SD-WAN expansion to improve latency and resilience?</t>
-  </si>
-  <si>
-    <t>Which purchase order is about WAN network modernization to reduce delay and improve stability?</t>
-  </si>
-  <si>
-    <t>Which contract governs managed cloud services for AWS and Azure with RTO/RPO requirements?</t>
-  </si>
-  <si>
-    <t>Which agreement covers cloud operations support with recovery time and recovery point targets?</t>
-  </si>
-  <si>
-    <t>Which purchase order supports infrastructure observability tooling for real-time metrics, alerting, and root-cause analysis?</t>
-  </si>
-  <si>
-    <t>Which purchase order is about system monitoring tools that provide live performance tracking, alerts, and issue diagnosis?</t>
+    <t>The purchase order related to cybersecurity monitoring and incident response services is PO-INF-003.</t>
+  </si>
+  <si>
+    <t>The purchase order for threat detection and security breach handling is PO-INF-003.</t>
+  </si>
+  <si>
+    <t>The contract is C-INF-008 – "Global Backup &amp; DR Agreement".</t>
+  </si>
+  <si>
+    <t>The agreement that covers data recovery planning, regular recovery testing, and financial consequences for failures is the “Global Backup &amp; DR Agreement” (contract number C-INF-008).</t>
+  </si>
+  <si>
+    <t>The contract is C-INF-004 – "Cloud Managed Services SLA".</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -935,6 +1134,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF31333F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8.25"/>
+      <color rgb="FF158237"/>
+      <name val="Source Code Pro"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -956,7 +1167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -967,6 +1178,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1270,57 +1484,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="45.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="28.8">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1332,81 +1546,81 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.8">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="28.8">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="B8" s="4"/>
     </row>
   </sheetData>
@@ -1416,89 +1630,123 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>12</v>
+      <c r="B3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="5" width="31.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="57.6">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="86.4">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="43.2">
+      <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="43.2">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="57.6">
+      <c r="A6" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1508,42 +1756,63 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="3" width="32.109375" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="43.2">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="43.2">
+      <c r="A3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="43.2">
+      <c r="A4" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="43.2">
+      <c r="A5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="43.2">
+      <c r="A6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="40.200000000000003">
+      <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>19</v>
+      <c r="B7" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>